<commit_message>
Final race data: judge complete (Opus 1926 + Grok 1926 + GPT 801 fail-fast); Results aggregated (261 official scores, 69 P2 stance deltas)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/official_20260619__Results聚合表.xlsx
+++ b/data/official_20260619__Results聚合表.xlsx
@@ -571,16 +571,16 @@
         <v>12</v>
       </c>
       <c r="F4" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G4" t="n">
         <v>2</v>
       </c>
       <c r="H4" t="n">
-        <v>2</v>
+        <v>2.059</v>
       </c>
       <c r="I4" t="n">
-        <v>0.545</v>
+        <v>0.6879999999999999</v>
       </c>
     </row>
     <row r="5">
@@ -799,7 +799,7 @@
         <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -2207,7 +2207,7 @@
         <v>3</v>
       </c>
       <c r="F47" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G47" t="n">
         <v>3</v>
@@ -2216,7 +2216,10 @@
         <v>3</v>
       </c>
       <c r="I47" t="n">
-        <v>0.667</v>
+        <v>0.833</v>
+      </c>
+      <c r="J47" t="n">
+        <v>1.667</v>
       </c>
     </row>
     <row r="48">
@@ -2244,13 +2247,13 @@
         <v>3</v>
       </c>
       <c r="F48" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G48" t="n">
         <v>3</v>
       </c>
       <c r="H48" t="n">
-        <v>3</v>
+        <v>2.833</v>
       </c>
       <c r="I48" t="n">
         <v>1</v>
@@ -2284,7 +2287,7 @@
         <v>3</v>
       </c>
       <c r="F49" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G49" t="n">
         <v>3</v>
@@ -2294,6 +2297,9 @@
       </c>
       <c r="I49" t="n">
         <v>1</v>
+      </c>
+      <c r="J49" t="n">
+        <v>0.667</v>
       </c>
     </row>
     <row r="50">
@@ -2321,7 +2327,7 @@
         <v>3</v>
       </c>
       <c r="F50" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G50" t="n">
         <v>3</v>
@@ -2361,7 +2367,7 @@
         <v>3</v>
       </c>
       <c r="F51" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G51" t="n">
         <v>3</v>
@@ -2370,7 +2376,7 @@
         <v>3</v>
       </c>
       <c r="I51" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="J51" t="n">
         <v>2</v>
@@ -2401,7 +2407,7 @@
         <v>3</v>
       </c>
       <c r="F52" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G52" t="n">
         <v>3</v>
@@ -2441,7 +2447,7 @@
         <v>3</v>
       </c>
       <c r="F53" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G53" t="n">
         <v>3</v>
@@ -2481,7 +2487,7 @@
         <v>3</v>
       </c>
       <c r="F54" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G54" t="n">
         <v>3</v>
@@ -2492,6 +2498,9 @@
       <c r="I54" t="n">
         <v>1</v>
       </c>
+      <c r="J54" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2518,13 +2527,13 @@
         <v>3</v>
       </c>
       <c r="F55" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G55" t="n">
         <v>3</v>
       </c>
       <c r="H55" t="n">
-        <v>3</v>
+        <v>2.667</v>
       </c>
       <c r="I55" t="n">
         <v>1</v>
@@ -2558,7 +2567,7 @@
         <v>12</v>
       </c>
       <c r="F56" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G56" t="n">
         <v>2</v>
@@ -2570,7 +2579,7 @@
         <v>1</v>
       </c>
       <c r="J56" t="n">
-        <v>1.667</v>
+        <v>1.933</v>
       </c>
     </row>
     <row r="57">
@@ -2598,19 +2607,19 @@
         <v>12</v>
       </c>
       <c r="F57" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G57" t="n">
         <v>2</v>
       </c>
       <c r="H57" t="n">
-        <v>1.833</v>
+        <v>1.917</v>
       </c>
       <c r="I57" t="n">
-        <v>0.75</v>
+        <v>0.833</v>
       </c>
       <c r="J57" t="n">
-        <v>0.75</v>
+        <v>1.643</v>
       </c>
     </row>
     <row r="58">
@@ -2638,19 +2647,19 @@
         <v>12</v>
       </c>
       <c r="F58" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G58" t="n">
         <v>2</v>
       </c>
       <c r="H58" t="n">
-        <v>1.75</v>
+        <v>2.083</v>
       </c>
       <c r="I58" t="n">
         <v>1</v>
       </c>
       <c r="J58" t="n">
-        <v>1.333</v>
+        <v>1.867</v>
       </c>
     </row>
     <row r="59">
@@ -2678,13 +2687,13 @@
         <v>12</v>
       </c>
       <c r="F59" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G59" t="n">
         <v>3</v>
       </c>
       <c r="H59" t="n">
-        <v>2.833</v>
+        <v>2.708</v>
       </c>
       <c r="I59" t="n">
         <v>1</v>
@@ -2718,19 +2727,19 @@
         <v>12</v>
       </c>
       <c r="F60" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G60" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="H60" t="n">
-        <v>2.5</v>
+        <v>2.542</v>
       </c>
       <c r="I60" t="n">
         <v>1</v>
       </c>
       <c r="J60" t="n">
-        <v>1.6</v>
+        <v>1.882</v>
       </c>
     </row>
     <row r="61">
@@ -2758,13 +2767,13 @@
         <v>12</v>
       </c>
       <c r="F61" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G61" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H61" t="n">
-        <v>2.583</v>
+        <v>2.458</v>
       </c>
       <c r="I61" t="n">
         <v>1</v>
@@ -2798,16 +2807,16 @@
         <v>3</v>
       </c>
       <c r="F62" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G62" t="n">
         <v>2</v>
       </c>
       <c r="H62" t="n">
-        <v>2.333</v>
+        <v>2.167</v>
       </c>
       <c r="I62" t="n">
-        <v>0.667</v>
+        <v>0.833</v>
       </c>
       <c r="J62" t="n">
         <v>2</v>
@@ -2838,19 +2847,19 @@
         <v>3</v>
       </c>
       <c r="F63" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G63" t="n">
         <v>2</v>
       </c>
       <c r="H63" t="n">
-        <v>2</v>
+        <v>2.167</v>
       </c>
       <c r="I63" t="n">
         <v>1</v>
       </c>
       <c r="J63" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="64">
@@ -2878,19 +2887,19 @@
         <v>3</v>
       </c>
       <c r="F64" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G64" t="n">
         <v>2</v>
       </c>
       <c r="H64" t="n">
-        <v>2</v>
+        <v>2.167</v>
       </c>
       <c r="I64" t="n">
         <v>1</v>
       </c>
       <c r="J64" t="n">
-        <v>1.667</v>
+        <v>1.833</v>
       </c>
     </row>
     <row r="65">
@@ -3155,16 +3164,19 @@
         <v>12</v>
       </c>
       <c r="F71" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G71" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="H71" t="n">
-        <v>2</v>
+        <v>2.417</v>
       </c>
       <c r="I71" t="n">
-        <v>0.636</v>
+        <v>0.826</v>
+      </c>
+      <c r="J71" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="72">
@@ -3192,19 +3204,19 @@
         <v>12</v>
       </c>
       <c r="F72" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G72" t="n">
         <v>2</v>
       </c>
       <c r="H72" t="n">
-        <v>1.833</v>
+        <v>2.208</v>
       </c>
       <c r="I72" t="n">
-        <v>0.667</v>
+        <v>0.833</v>
       </c>
       <c r="J72" t="n">
-        <v>0</v>
+        <v>1.75</v>
       </c>
     </row>
     <row r="73">
@@ -3232,16 +3244,19 @@
         <v>12</v>
       </c>
       <c r="F73" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G73" t="n">
         <v>2</v>
       </c>
       <c r="H73" t="n">
-        <v>1.417</v>
+        <v>1.667</v>
       </c>
       <c r="I73" t="n">
-        <v>0.833</v>
+        <v>0.875</v>
+      </c>
+      <c r="J73" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="74">
@@ -3269,13 +3284,13 @@
         <v>12</v>
       </c>
       <c r="F74" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G74" t="n">
         <v>0</v>
       </c>
       <c r="H74" t="n">
-        <v>0.167</v>
+        <v>0.083</v>
       </c>
       <c r="I74" t="n">
         <v>0</v>
@@ -3306,19 +3321,19 @@
         <v>12</v>
       </c>
       <c r="F75" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G75" t="n">
         <v>0</v>
       </c>
       <c r="H75" t="n">
-        <v>0.75</v>
+        <v>0.375</v>
       </c>
       <c r="I75" t="n">
         <v>0</v>
       </c>
       <c r="J75" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="76">
@@ -3346,13 +3361,13 @@
         <v>12</v>
       </c>
       <c r="F76" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G76" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H76" t="n">
-        <v>1.417</v>
+        <v>0.708</v>
       </c>
       <c r="I76" t="n">
         <v>0</v>
@@ -3386,7 +3401,7 @@
         <v>3</v>
       </c>
       <c r="F77" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G77" t="n">
         <v>0</v>
@@ -3423,7 +3438,7 @@
         <v>3</v>
       </c>
       <c r="F78" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G78" t="n">
         <v>0</v>
@@ -3460,7 +3475,7 @@
         <v>3</v>
       </c>
       <c r="F79" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G79" t="n">
         <v>0</v>
@@ -3497,7 +3512,7 @@
         <v>3</v>
       </c>
       <c r="F80" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G80" t="n">
         <v>1</v>
@@ -3537,7 +3552,7 @@
         <v>3</v>
       </c>
       <c r="F81" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G81" t="n">
         <v>0</v>
@@ -3577,7 +3592,7 @@
         <v>3</v>
       </c>
       <c r="F82" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G82" t="n">
         <v>1</v>
@@ -3842,16 +3857,19 @@
         <v>12</v>
       </c>
       <c r="F89" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G89" t="n">
         <v>2</v>
       </c>
       <c r="H89" t="n">
-        <v>2.083</v>
+        <v>2.292</v>
       </c>
       <c r="I89" t="n">
-        <v>0</v>
+        <v>0.55</v>
+      </c>
+      <c r="J89" t="n">
+        <v>1.5</v>
       </c>
     </row>
     <row r="90">
@@ -3879,16 +3897,19 @@
         <v>12</v>
       </c>
       <c r="F90" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G90" t="n">
         <v>3</v>
       </c>
       <c r="H90" t="n">
-        <v>2.75</v>
+        <v>2.833</v>
       </c>
       <c r="I90" t="n">
-        <v>0.333</v>
+        <v>0.667</v>
+      </c>
+      <c r="J90" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="91">
@@ -3916,16 +3937,19 @@
         <v>12</v>
       </c>
       <c r="F91" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G91" t="n">
         <v>2</v>
       </c>
       <c r="H91" t="n">
-        <v>1.833</v>
+        <v>2</v>
       </c>
       <c r="I91" t="n">
-        <v>0.455</v>
+        <v>0.696</v>
+      </c>
+      <c r="J91" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="92">
@@ -3953,13 +3977,13 @@
         <v>12</v>
       </c>
       <c r="F92" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G92" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H92" t="n">
-        <v>1.417</v>
+        <v>0.792</v>
       </c>
       <c r="I92" t="n">
         <v>0.417</v>
@@ -3990,13 +4014,13 @@
         <v>12</v>
       </c>
       <c r="F93" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G93" t="n">
         <v>0</v>
       </c>
       <c r="H93" t="n">
-        <v>0.083</v>
+        <v>0.042</v>
       </c>
       <c r="I93" t="n">
         <v>0</v>
@@ -4027,16 +4051,16 @@
         <v>12</v>
       </c>
       <c r="F94" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G94" t="n">
         <v>0</v>
       </c>
       <c r="H94" t="n">
-        <v>0.583</v>
+        <v>0.292</v>
       </c>
       <c r="I94" t="n">
-        <v>0.182</v>
+        <v>0.167</v>
       </c>
       <c r="J94" t="n">
         <v>0</v>
@@ -4067,7 +4091,7 @@
         <v>3</v>
       </c>
       <c r="F95" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G95" t="n">
         <v>0</v>
@@ -4104,7 +4128,7 @@
         <v>3</v>
       </c>
       <c r="F96" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G96" t="n">
         <v>0</v>
@@ -4141,7 +4165,7 @@
         <v>3</v>
       </c>
       <c r="F97" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G97" t="n">
         <v>0</v>
@@ -4415,7 +4439,7 @@
         <v>12</v>
       </c>
       <c r="F104" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G104" t="n">
         <v>2</v>
@@ -4424,7 +4448,10 @@
         <v>2.25</v>
       </c>
       <c r="I104" t="n">
-        <v>0.8179999999999999</v>
+        <v>0.87</v>
+      </c>
+      <c r="J104" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="105">
@@ -4452,16 +4479,16 @@
         <v>12</v>
       </c>
       <c r="F105" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G105" t="n">
         <v>2.5</v>
       </c>
       <c r="H105" t="n">
-        <v>2.5</v>
+        <v>2.417</v>
       </c>
       <c r="I105" t="n">
-        <v>0.833</v>
+        <v>0.917</v>
       </c>
       <c r="J105" t="n">
         <v>2</v>
@@ -4492,19 +4519,19 @@
         <v>12</v>
       </c>
       <c r="F106" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G106" t="n">
         <v>2</v>
       </c>
       <c r="H106" t="n">
-        <v>1.5</v>
+        <v>1.826</v>
       </c>
       <c r="I106" t="n">
-        <v>0.917</v>
+        <v>0.913</v>
       </c>
       <c r="J106" t="n">
-        <v>2</v>
+        <v>1.667</v>
       </c>
     </row>
     <row r="107">
@@ -4532,19 +4559,19 @@
         <v>12</v>
       </c>
       <c r="F107" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="G107" t="n">
         <v>2</v>
       </c>
       <c r="H107" t="n">
-        <v>2.083</v>
+        <v>1.85</v>
       </c>
       <c r="I107" t="n">
         <v>1</v>
       </c>
       <c r="J107" t="n">
-        <v>1</v>
+        <v>1.75</v>
       </c>
     </row>
     <row r="108">
@@ -4572,13 +4599,13 @@
         <v>12</v>
       </c>
       <c r="F108" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G108" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H108" t="n">
-        <v>2.583</v>
+        <v>2.458</v>
       </c>
       <c r="I108" t="n">
         <v>1</v>
@@ -4612,13 +4639,13 @@
         <v>12</v>
       </c>
       <c r="F109" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G109" t="n">
         <v>2</v>
       </c>
       <c r="H109" t="n">
-        <v>2.333</v>
+        <v>2.167</v>
       </c>
       <c r="I109" t="n">
         <v>1</v>
@@ -4652,16 +4679,19 @@
         <v>3</v>
       </c>
       <c r="F110" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G110" t="n">
         <v>2</v>
       </c>
       <c r="H110" t="n">
-        <v>1.333</v>
+        <v>1.667</v>
       </c>
       <c r="I110" t="n">
         <v>1</v>
+      </c>
+      <c r="J110" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="111">
@@ -4689,16 +4719,19 @@
         <v>3</v>
       </c>
       <c r="F111" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G111" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H111" t="n">
-        <v>0.667</v>
+        <v>1</v>
       </c>
       <c r="I111" t="n">
         <v>1</v>
+      </c>
+      <c r="J111" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="112">
@@ -4726,7 +4759,7 @@
         <v>3</v>
       </c>
       <c r="F112" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G112" t="n">
         <v>2</v>
@@ -4737,6 +4770,9 @@
       <c r="I112" t="n">
         <v>1</v>
       </c>
+      <c r="J112" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -5915,7 +5951,7 @@
         <v>12</v>
       </c>
       <c r="F143" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G143" t="n">
         <v>2</v>
@@ -5924,10 +5960,10 @@
         <v>2.167</v>
       </c>
       <c r="I143" t="n">
-        <v>0.833</v>
+        <v>0.917</v>
       </c>
       <c r="J143" t="n">
-        <v>1</v>
+        <v>1.857</v>
       </c>
     </row>
     <row r="144">
@@ -5955,19 +5991,19 @@
         <v>12</v>
       </c>
       <c r="F144" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G144" t="n">
         <v>3</v>
       </c>
       <c r="H144" t="n">
-        <v>2.75</v>
+        <v>2.875</v>
       </c>
       <c r="I144" t="n">
         <v>1</v>
       </c>
       <c r="J144" t="n">
-        <v>0</v>
+        <v>1.077</v>
       </c>
     </row>
     <row r="145">
@@ -6035,13 +6071,13 @@
         <v>12</v>
       </c>
       <c r="F146" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G146" t="n">
         <v>3</v>
       </c>
       <c r="H146" t="n">
-        <v>2.917</v>
+        <v>2.958</v>
       </c>
       <c r="I146" t="n">
         <v>1</v>
@@ -6075,13 +6111,13 @@
         <v>12</v>
       </c>
       <c r="F147" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G147" t="n">
         <v>3</v>
       </c>
       <c r="H147" t="n">
-        <v>2.667</v>
+        <v>2.625</v>
       </c>
       <c r="I147" t="n">
         <v>1</v>
@@ -6155,19 +6191,19 @@
         <v>3</v>
       </c>
       <c r="F149" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G149" t="n">
         <v>2</v>
       </c>
       <c r="H149" t="n">
-        <v>1.667</v>
+        <v>1.833</v>
       </c>
       <c r="I149" t="n">
-        <v>0.333</v>
+        <v>0.667</v>
       </c>
       <c r="J149" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="150">
@@ -6195,19 +6231,19 @@
         <v>3</v>
       </c>
       <c r="F150" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G150" t="n">
         <v>2</v>
       </c>
       <c r="H150" t="n">
-        <v>2.25</v>
+        <v>2.167</v>
       </c>
       <c r="I150" t="n">
         <v>1</v>
       </c>
       <c r="J150" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="151">
@@ -6512,16 +6548,19 @@
         <v>12</v>
       </c>
       <c r="F158" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G158" t="n">
         <v>2</v>
       </c>
       <c r="H158" t="n">
-        <v>1.333</v>
+        <v>1.542</v>
       </c>
       <c r="I158" t="n">
-        <v>0.333</v>
+        <v>0.619</v>
+      </c>
+      <c r="J158" t="n">
+        <v>1.667</v>
       </c>
     </row>
     <row r="159">
@@ -6549,16 +6588,19 @@
         <v>12</v>
       </c>
       <c r="F159" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G159" t="n">
         <v>2</v>
       </c>
       <c r="H159" t="n">
-        <v>1.667</v>
+        <v>2.083</v>
       </c>
       <c r="I159" t="n">
-        <v>0.727</v>
+        <v>0.87</v>
+      </c>
+      <c r="J159" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="160">
@@ -6586,19 +6628,19 @@
         <v>12</v>
       </c>
       <c r="F160" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G160" t="n">
         <v>2</v>
       </c>
       <c r="H160" t="n">
-        <v>1.75</v>
+        <v>2</v>
       </c>
       <c r="I160" t="n">
-        <v>0.8179999999999999</v>
+        <v>0.913</v>
       </c>
       <c r="J160" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="161">
@@ -6626,16 +6668,16 @@
         <v>12</v>
       </c>
       <c r="F161" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G161" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="H161" t="n">
-        <v>1.917</v>
+        <v>1.25</v>
       </c>
       <c r="I161" t="n">
-        <v>0.083</v>
+        <v>0.062</v>
       </c>
     </row>
     <row r="162">
@@ -6663,16 +6705,19 @@
         <v>12</v>
       </c>
       <c r="F162" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G162" t="n">
         <v>2</v>
       </c>
       <c r="H162" t="n">
-        <v>1.917</v>
+        <v>1.25</v>
       </c>
       <c r="I162" t="n">
-        <v>0.167</v>
+        <v>0.125</v>
+      </c>
+      <c r="J162" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="163">
@@ -6700,16 +6745,19 @@
         <v>12</v>
       </c>
       <c r="F163" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G163" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="H163" t="n">
-        <v>2.167</v>
+        <v>1.208</v>
       </c>
       <c r="I163" t="n">
-        <v>0.364</v>
+        <v>0.267</v>
+      </c>
+      <c r="J163" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="164">
@@ -6737,7 +6785,7 @@
         <v>3</v>
       </c>
       <c r="F164" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G164" t="n">
         <v>0</v>
@@ -6774,7 +6822,7 @@
         <v>3</v>
       </c>
       <c r="F165" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G165" t="n">
         <v>0</v>
@@ -6811,7 +6859,7 @@
         <v>3</v>
       </c>
       <c r="F166" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G166" t="n">
         <v>0</v>
@@ -7544,16 +7592,16 @@
         <v>12</v>
       </c>
       <c r="F185" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G185" t="n">
         <v>1</v>
       </c>
       <c r="H185" t="n">
-        <v>1</v>
+        <v>1.375</v>
       </c>
       <c r="I185" t="n">
-        <v>1</v>
+        <v>0.643</v>
       </c>
       <c r="J185" t="n">
         <v>1.2</v>
@@ -7584,16 +7632,16 @@
         <v>12</v>
       </c>
       <c r="F186" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G186" t="n">
         <v>2</v>
       </c>
       <c r="H186" t="n">
-        <v>2</v>
+        <v>2.042</v>
       </c>
       <c r="I186" t="n">
-        <v>1</v>
+        <v>0.652</v>
       </c>
       <c r="J186" t="n">
         <v>1</v>
@@ -7624,19 +7672,19 @@
         <v>3</v>
       </c>
       <c r="F187" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G187" t="n">
         <v>2</v>
       </c>
       <c r="H187" t="n">
-        <v>2</v>
+        <v>2.167</v>
       </c>
       <c r="I187" t="n">
         <v>1</v>
       </c>
       <c r="J187" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="188">
@@ -7664,13 +7712,13 @@
         <v>12</v>
       </c>
       <c r="F188" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G188" t="n">
         <v>2</v>
       </c>
       <c r="H188" t="n">
-        <v>1.7</v>
+        <v>2.227</v>
       </c>
       <c r="I188" t="n">
         <v>1</v>
@@ -7704,13 +7752,13 @@
         <v>12</v>
       </c>
       <c r="F189" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G189" t="n">
         <v>2</v>
       </c>
       <c r="H189" t="n">
-        <v>2</v>
+        <v>2.333</v>
       </c>
       <c r="I189" t="n">
         <v>1</v>
@@ -7744,13 +7792,13 @@
         <v>3</v>
       </c>
       <c r="F190" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G190" t="n">
         <v>3</v>
       </c>
       <c r="H190" t="n">
-        <v>2.667</v>
+        <v>2.833</v>
       </c>
       <c r="I190" t="n">
         <v>1</v>
@@ -7784,7 +7832,7 @@
         <v>12</v>
       </c>
       <c r="F191" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G191" t="n">
         <v>2</v>
@@ -7821,19 +7869,19 @@
         <v>12</v>
       </c>
       <c r="F192" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G192" t="n">
         <v>2</v>
       </c>
       <c r="H192" t="n">
-        <v>2</v>
+        <v>1.769</v>
       </c>
       <c r="I192" t="n">
         <v>1</v>
       </c>
       <c r="J192" t="n">
-        <v>1</v>
+        <v>0.667</v>
       </c>
     </row>
     <row r="193">
@@ -7861,19 +7909,19 @@
         <v>12</v>
       </c>
       <c r="F193" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G193" t="n">
         <v>2</v>
       </c>
       <c r="H193" t="n">
-        <v>1.917</v>
+        <v>1.87</v>
       </c>
       <c r="I193" t="n">
         <v>1</v>
       </c>
       <c r="J193" t="n">
-        <v>1</v>
+        <v>1.333</v>
       </c>
     </row>
     <row r="194">
@@ -7901,19 +7949,19 @@
         <v>12</v>
       </c>
       <c r="F194" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G194" t="n">
         <v>1</v>
       </c>
       <c r="H194" t="n">
-        <v>1.167</v>
+        <v>1.083</v>
       </c>
       <c r="I194" t="n">
+        <v>0.708</v>
+      </c>
+      <c r="J194" t="n">
         <v>0.5</v>
-      </c>
-      <c r="J194" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="195">
@@ -7941,7 +7989,13 @@
         <v>12</v>
       </c>
       <c r="F195" t="n">
-        <v>12</v>
+        <v>24</v>
+      </c>
+      <c r="G195" t="n">
+        <v>2</v>
+      </c>
+      <c r="H195" t="n">
+        <v>2</v>
       </c>
       <c r="I195" t="n">
         <v>1</v>
@@ -7972,19 +8026,19 @@
         <v>12</v>
       </c>
       <c r="F196" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G196" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H196" t="n">
-        <v>1.417</v>
+        <v>1.708</v>
       </c>
       <c r="I196" t="n">
-        <v>0.917</v>
+        <v>0.958</v>
       </c>
       <c r="J196" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="197">
@@ -8012,13 +8066,13 @@
         <v>3</v>
       </c>
       <c r="F197" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G197" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="H197" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="I197" t="n">
         <v>1</v>
@@ -8049,7 +8103,13 @@
         <v>3</v>
       </c>
       <c r="F198" t="n">
-        <v>3</v>
+        <v>6</v>
+      </c>
+      <c r="G198" t="n">
+        <v>2</v>
+      </c>
+      <c r="H198" t="n">
+        <v>2</v>
       </c>
       <c r="I198" t="n">
         <v>1</v>
@@ -8080,16 +8140,19 @@
         <v>3</v>
       </c>
       <c r="F199" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G199" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="H199" t="n">
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="I199" t="n">
-        <v>0.75</v>
+        <v>0.833</v>
+      </c>
+      <c r="J199" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="200">
@@ -8117,13 +8180,13 @@
         <v>12</v>
       </c>
       <c r="F200" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G200" t="n">
         <v>2</v>
       </c>
       <c r="H200" t="n">
-        <v>1.917</v>
+        <v>1.833</v>
       </c>
       <c r="I200" t="n">
         <v>1</v>
@@ -8154,19 +8217,19 @@
         <v>12</v>
       </c>
       <c r="F201" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G201" t="n">
         <v>1</v>
       </c>
       <c r="H201" t="n">
-        <v>1.333</v>
+        <v>1.267</v>
       </c>
       <c r="I201" t="n">
-        <v>1</v>
+        <v>0.9379999999999999</v>
       </c>
       <c r="J201" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="202">
@@ -8194,16 +8257,16 @@
         <v>12</v>
       </c>
       <c r="F202" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G202" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="H202" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="I202" t="n">
-        <v>1</v>
+        <v>0.958</v>
       </c>
       <c r="J202" t="n">
         <v>1</v>
@@ -8234,13 +8297,13 @@
         <v>12</v>
       </c>
       <c r="F203" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G203" t="n">
         <v>2</v>
       </c>
       <c r="H203" t="n">
-        <v>2</v>
+        <v>2.25</v>
       </c>
       <c r="I203" t="n">
         <v>1</v>
@@ -8271,13 +8334,13 @@
         <v>12</v>
       </c>
       <c r="F204" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G204" t="n">
         <v>2</v>
       </c>
       <c r="H204" t="n">
-        <v>2</v>
+        <v>2.125</v>
       </c>
       <c r="I204" t="n">
         <v>1</v>
@@ -8308,13 +8371,13 @@
         <v>12</v>
       </c>
       <c r="F205" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G205" t="n">
         <v>2</v>
       </c>
       <c r="H205" t="n">
-        <v>2</v>
+        <v>2.208</v>
       </c>
       <c r="I205" t="n">
         <v>1</v>
@@ -8345,13 +8408,13 @@
         <v>3</v>
       </c>
       <c r="F206" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G206" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H206" t="n">
-        <v>2.333</v>
+        <v>2.667</v>
       </c>
       <c r="I206" t="n">
         <v>1</v>
@@ -8382,16 +8445,16 @@
         <v>3</v>
       </c>
       <c r="F207" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G207" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H207" t="n">
-        <v>2</v>
+        <v>2.75</v>
       </c>
       <c r="I207" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="208">
@@ -8419,13 +8482,13 @@
         <v>3</v>
       </c>
       <c r="F208" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G208" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="H208" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="I208" t="n">
         <v>1</v>
@@ -8456,19 +8519,19 @@
         <v>12</v>
       </c>
       <c r="F209" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G209" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="H209" t="n">
-        <v>2.167</v>
+        <v>2.292</v>
       </c>
       <c r="I209" t="n">
-        <v>0.917</v>
+        <v>0.609</v>
       </c>
       <c r="J209" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="210">
@@ -8496,16 +8559,16 @@
         <v>12</v>
       </c>
       <c r="F210" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G210" t="n">
         <v>3</v>
       </c>
       <c r="H210" t="n">
-        <v>3</v>
+        <v>2.769</v>
       </c>
       <c r="I210" t="n">
-        <v>1</v>
+        <v>0.846</v>
       </c>
     </row>
     <row r="211">
@@ -8533,16 +8596,16 @@
         <v>12</v>
       </c>
       <c r="F211" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G211" t="n">
         <v>3</v>
       </c>
       <c r="H211" t="n">
-        <v>2.667</v>
+        <v>2.792</v>
       </c>
       <c r="I211" t="n">
-        <v>1</v>
+        <v>0.792</v>
       </c>
       <c r="J211" t="n">
         <v>2</v>
@@ -8573,7 +8636,7 @@
         <v>12</v>
       </c>
       <c r="F212" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G212" t="n">
         <v>0</v>
@@ -8582,7 +8645,7 @@
         <v>0</v>
       </c>
       <c r="I212" t="n">
-        <v>0.7</v>
+        <v>0.318</v>
       </c>
       <c r="J212" t="n">
         <v>0</v>
@@ -8613,7 +8676,7 @@
         <v>12</v>
       </c>
       <c r="F213" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G213" t="n">
         <v>0</v>
@@ -8622,7 +8685,7 @@
         <v>0</v>
       </c>
       <c r="I213" t="n">
-        <v>0.667</v>
+        <v>0.2</v>
       </c>
       <c r="J213" t="n">
         <v>0</v>
@@ -8653,16 +8716,16 @@
         <v>12</v>
       </c>
       <c r="F214" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G214" t="n">
         <v>0</v>
       </c>
       <c r="H214" t="n">
-        <v>0.25</v>
+        <v>0.125</v>
       </c>
       <c r="I214" t="n">
-        <v>0.417</v>
+        <v>0.292</v>
       </c>
       <c r="J214" t="n">
         <v>0</v>
@@ -8693,7 +8756,7 @@
         <v>3</v>
       </c>
       <c r="F215" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G215" t="n">
         <v>0</v>
@@ -8702,7 +8765,7 @@
         <v>0</v>
       </c>
       <c r="I215" t="n">
-        <v>0.667</v>
+        <v>0.333</v>
       </c>
     </row>
     <row r="216">
@@ -8730,7 +8793,16 @@
         <v>3</v>
       </c>
       <c r="F216" t="n">
-        <v>3</v>
+        <v>6</v>
+      </c>
+      <c r="G216" t="n">
+        <v>0</v>
+      </c>
+      <c r="H216" t="n">
+        <v>0</v>
+      </c>
+      <c r="I216" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="217">
@@ -8758,7 +8830,7 @@
         <v>3</v>
       </c>
       <c r="F217" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G217" t="n">
         <v>0</v>
@@ -8767,7 +8839,7 @@
         <v>0</v>
       </c>
       <c r="I217" t="n">
-        <v>0.667</v>
+        <v>0.333</v>
       </c>
     </row>
     <row r="218">
@@ -10539,7 +10611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10657,13 +10729,13 @@
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>2.059</v>
       </c>
       <c r="F4" t="n">
         <v>0.75</v>
       </c>
       <c r="G4" t="n">
-        <v>-1.25</v>
+        <v>-1.309</v>
       </c>
     </row>
     <row r="5">
@@ -11034,13 +11106,13 @@
         <v>2.667</v>
       </c>
       <c r="E17" t="n">
-        <v>3</v>
+        <v>2.833</v>
       </c>
       <c r="F17" t="n">
         <v>3</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>0.167</v>
       </c>
     </row>
     <row r="18">
@@ -11060,7 +11132,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>3</v>
+        <v>2.667</v>
       </c>
       <c r="E18" t="n">
         <v>3</v>
@@ -11089,16 +11161,16 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>2.333</v>
+        <v>2.167</v>
       </c>
       <c r="E19" t="n">
         <v>2.167</v>
       </c>
       <c r="F19" t="n">
-        <v>2.833</v>
+        <v>2.708</v>
       </c>
       <c r="G19" t="n">
-        <v>0.666</v>
+        <v>0.541</v>
       </c>
     </row>
     <row r="20">
@@ -11118,16 +11190,16 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>2</v>
+        <v>2.167</v>
       </c>
       <c r="E20" t="n">
-        <v>1.833</v>
+        <v>1.917</v>
       </c>
       <c r="F20" t="n">
-        <v>2.5</v>
+        <v>2.542</v>
       </c>
       <c r="G20" t="n">
-        <v>0.667</v>
+        <v>0.625</v>
       </c>
     </row>
     <row r="21">
@@ -11147,16 +11219,16 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>2</v>
+        <v>2.167</v>
       </c>
       <c r="E21" t="n">
-        <v>1.75</v>
+        <v>2.083</v>
       </c>
       <c r="F21" t="n">
-        <v>2.583</v>
+        <v>2.458</v>
       </c>
       <c r="G21" t="n">
-        <v>0.833</v>
+        <v>0.375</v>
       </c>
     </row>
     <row r="22">
@@ -11179,13 +11251,13 @@
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>2.417</v>
       </c>
       <c r="F22" t="n">
-        <v>0.167</v>
+        <v>0.083</v>
       </c>
       <c r="G22" t="n">
-        <v>-1.833</v>
+        <v>-2.334</v>
       </c>
     </row>
     <row r="23">
@@ -11208,13 +11280,13 @@
         <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>1.833</v>
+        <v>2.208</v>
       </c>
       <c r="F23" t="n">
-        <v>0.75</v>
+        <v>0.375</v>
       </c>
       <c r="G23" t="n">
-        <v>-1.083</v>
+        <v>-1.833</v>
       </c>
     </row>
     <row r="24">
@@ -11237,13 +11309,13 @@
         <v>0</v>
       </c>
       <c r="E24" t="n">
-        <v>1.417</v>
+        <v>1.667</v>
       </c>
       <c r="F24" t="n">
-        <v>1.417</v>
+        <v>0.708</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>-0.959</v>
       </c>
     </row>
     <row r="25">
@@ -11266,13 +11338,13 @@
         <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>2.083</v>
+        <v>2.292</v>
       </c>
       <c r="F25" t="n">
-        <v>1.417</v>
+        <v>0.792</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.666</v>
+        <v>-1.5</v>
       </c>
     </row>
     <row r="26">
@@ -11295,13 +11367,13 @@
         <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>2.75</v>
+        <v>2.833</v>
       </c>
       <c r="F26" t="n">
-        <v>0.083</v>
+        <v>0.042</v>
       </c>
       <c r="G26" t="n">
-        <v>-2.667</v>
+        <v>-2.791</v>
       </c>
     </row>
     <row r="27">
@@ -11324,13 +11396,13 @@
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>1.833</v>
+        <v>2</v>
       </c>
       <c r="F27" t="n">
-        <v>0.583</v>
+        <v>0.292</v>
       </c>
       <c r="G27" t="n">
-        <v>-1.25</v>
+        <v>-1.708</v>
       </c>
     </row>
     <row r="28">
@@ -11408,16 +11480,16 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1.333</v>
+        <v>1.667</v>
       </c>
       <c r="E30" t="n">
         <v>2.25</v>
       </c>
       <c r="F30" t="n">
-        <v>2.083</v>
+        <v>1.85</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.167</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="31">
@@ -11437,16 +11509,16 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.667</v>
+        <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>2.5</v>
+        <v>2.417</v>
       </c>
       <c r="F31" t="n">
-        <v>2.583</v>
+        <v>2.458</v>
       </c>
       <c r="G31" t="n">
-        <v>0.083</v>
+        <v>0.041</v>
       </c>
     </row>
     <row r="32">
@@ -11469,13 +11541,13 @@
         <v>1.333</v>
       </c>
       <c r="E32" t="n">
-        <v>1.5</v>
+        <v>1.826</v>
       </c>
       <c r="F32" t="n">
-        <v>2.333</v>
+        <v>2.167</v>
       </c>
       <c r="G32" t="n">
-        <v>0.833</v>
+        <v>0.341</v>
       </c>
     </row>
     <row r="33">
@@ -11756,16 +11828,16 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>1.667</v>
+        <v>1.833</v>
       </c>
       <c r="E42" t="n">
         <v>2.167</v>
       </c>
       <c r="F42" t="n">
-        <v>2.917</v>
+        <v>2.958</v>
       </c>
       <c r="G42" t="n">
-        <v>0.75</v>
+        <v>0.791</v>
       </c>
     </row>
     <row r="43">
@@ -11785,16 +11857,16 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>2.25</v>
+        <v>2.167</v>
       </c>
       <c r="E43" t="n">
-        <v>2.75</v>
+        <v>2.875</v>
       </c>
       <c r="F43" t="n">
-        <v>2.667</v>
+        <v>2.625</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.083</v>
+        <v>-0.25</v>
       </c>
     </row>
     <row r="44">
@@ -11846,13 +11918,13 @@
         <v>0</v>
       </c>
       <c r="E45" t="n">
-        <v>1.333</v>
+        <v>1.542</v>
       </c>
       <c r="F45" t="n">
-        <v>1.917</v>
+        <v>1.25</v>
       </c>
       <c r="G45" t="n">
-        <v>0.584</v>
+        <v>-0.292</v>
       </c>
     </row>
     <row r="46">
@@ -11875,13 +11947,13 @@
         <v>0</v>
       </c>
       <c r="E46" t="n">
-        <v>1.667</v>
+        <v>2.083</v>
       </c>
       <c r="F46" t="n">
-        <v>1.917</v>
+        <v>1.25</v>
       </c>
       <c r="G46" t="n">
-        <v>0.25</v>
+        <v>-0.833</v>
       </c>
     </row>
     <row r="47">
@@ -11904,13 +11976,13 @@
         <v>0</v>
       </c>
       <c r="E47" t="n">
-        <v>1.75</v>
+        <v>2</v>
       </c>
       <c r="F47" t="n">
-        <v>2.167</v>
+        <v>1.208</v>
       </c>
       <c r="G47" t="n">
-        <v>0.417</v>
+        <v>-0.792</v>
       </c>
     </row>
     <row r="48">
@@ -12017,16 +12089,16 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>2</v>
+        <v>2.167</v>
       </c>
       <c r="E51" t="n">
-        <v>1</v>
+        <v>1.375</v>
       </c>
       <c r="F51" t="n">
-        <v>2</v>
+        <v>2.042</v>
       </c>
       <c r="G51" t="n">
-        <v>1</v>
+        <v>0.667</v>
       </c>
     </row>
     <row r="52">
@@ -12046,16 +12118,16 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>2.667</v>
+        <v>2.833</v>
       </c>
       <c r="E52" t="n">
-        <v>1.7</v>
+        <v>2.227</v>
       </c>
       <c r="F52" t="n">
-        <v>2</v>
+        <v>2.333</v>
       </c>
       <c r="G52" t="n">
-        <v>0.3</v>
+        <v>0.106</v>
       </c>
     </row>
     <row r="53">
@@ -12075,16 +12147,16 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="E53" t="n">
         <v>2</v>
       </c>
       <c r="F53" t="n">
-        <v>1.167</v>
+        <v>1.083</v>
       </c>
       <c r="G53" t="n">
-        <v>-0.833</v>
+        <v>-0.917</v>
       </c>
     </row>
     <row r="54">
@@ -12100,20 +12172,20 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>zh-Hant</t>
+          <t>zh-Hans</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>1.25</v>
+        <v>2</v>
       </c>
       <c r="E54" t="n">
-        <v>1.917</v>
+        <v>1.769</v>
       </c>
       <c r="F54" t="n">
-        <v>1.417</v>
+        <v>2</v>
       </c>
       <c r="G54" t="n">
-        <v>-0.5</v>
+        <v>0.231</v>
       </c>
     </row>
     <row r="55">
@@ -12124,25 +12196,25 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>T14</t>
+          <t>T13</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>zh-Hant</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>2.333</v>
+        <v>1.5</v>
       </c>
       <c r="E55" t="n">
-        <v>1.917</v>
+        <v>1.87</v>
       </c>
       <c r="F55" t="n">
-        <v>2</v>
+        <v>1.708</v>
       </c>
       <c r="G55" t="n">
-        <v>0.083</v>
+        <v>-0.162</v>
       </c>
     </row>
     <row r="56">
@@ -12158,20 +12230,20 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>zh-Hans</t>
+          <t>en</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>2</v>
+        <v>2.667</v>
       </c>
       <c r="E56" t="n">
-        <v>1.333</v>
+        <v>1.833</v>
       </c>
       <c r="F56" t="n">
-        <v>2</v>
+        <v>2.25</v>
       </c>
       <c r="G56" t="n">
-        <v>0.667</v>
+        <v>0.417</v>
       </c>
     </row>
     <row r="57">
@@ -12187,20 +12259,20 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>zh-Hant</t>
+          <t>zh-Hans</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>2</v>
+        <v>2.75</v>
       </c>
       <c r="E57" t="n">
-        <v>1.5</v>
+        <v>1.267</v>
       </c>
       <c r="F57" t="n">
-        <v>2</v>
+        <v>2.125</v>
       </c>
       <c r="G57" t="n">
-        <v>0.5</v>
+        <v>0.858</v>
       </c>
     </row>
     <row r="58">
@@ -12211,25 +12283,25 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T14</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>zh-Hant</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="E58" t="n">
-        <v>2.167</v>
+        <v>1</v>
       </c>
       <c r="F58" t="n">
-        <v>0</v>
+        <v>2.208</v>
       </c>
       <c r="G58" t="n">
-        <v>-2.167</v>
+        <v>1.208</v>
       </c>
     </row>
     <row r="59">
@@ -12245,17 +12317,20 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>zh-Hans</t>
-        </is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>0</v>
       </c>
       <c r="E59" t="n">
-        <v>3</v>
+        <v>2.292</v>
       </c>
       <c r="F59" t="n">
         <v>0</v>
       </c>
       <c r="G59" t="n">
-        <v>-3</v>
+        <v>-2.292</v>
       </c>
     </row>
     <row r="60">
@@ -12271,20 +12346,20 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>zh-Hant</t>
+          <t>zh-Hans</t>
         </is>
       </c>
       <c r="D60" t="n">
         <v>0</v>
       </c>
       <c r="E60" t="n">
-        <v>2.667</v>
+        <v>2.769</v>
       </c>
       <c r="F60" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="G60" t="n">
-        <v>-2.417</v>
+        <v>-2.769</v>
       </c>
     </row>
     <row r="61">
@@ -12295,25 +12370,25 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>T5flip</t>
+          <t>T15</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>zh-Hant</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E61" t="n">
-        <v>2.5</v>
+        <v>2.792</v>
       </c>
       <c r="F61" t="n">
-        <v>2.833</v>
+        <v>0.125</v>
       </c>
       <c r="G61" t="n">
-        <v>0.333</v>
+        <v>-2.667</v>
       </c>
     </row>
     <row r="62">
@@ -12329,20 +12404,20 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>zh-Hans</t>
+          <t>en</t>
         </is>
       </c>
       <c r="D62" t="n">
         <v>3</v>
       </c>
       <c r="E62" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="F62" t="n">
-        <v>2</v>
+        <v>2.833</v>
       </c>
       <c r="G62" t="n">
-        <v>0</v>
+        <v>0.333</v>
       </c>
     </row>
     <row r="63">
@@ -12358,20 +12433,20 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>zh-Hant</t>
+          <t>zh-Hans</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>2.667</v>
+        <v>3</v>
       </c>
       <c r="E63" t="n">
-        <v>1.667</v>
+        <v>2</v>
       </c>
       <c r="F63" t="n">
-        <v>2.833</v>
+        <v>2</v>
       </c>
       <c r="G63" t="n">
-        <v>1.166</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
@@ -12382,25 +12457,25 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>T6flip</t>
+          <t>T5flip</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>zh-Hant</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>2.167</v>
+        <v>2.667</v>
       </c>
       <c r="E64" t="n">
-        <v>2.125</v>
+        <v>1.667</v>
       </c>
       <c r="F64" t="n">
-        <v>2.042</v>
+        <v>2.833</v>
       </c>
       <c r="G64" t="n">
-        <v>-0.083</v>
+        <v>1.166</v>
       </c>
     </row>
     <row r="65">
@@ -12416,20 +12491,20 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>zh-Hans</t>
+          <t>en</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>2</v>
+        <v>2.167</v>
       </c>
       <c r="E65" t="n">
-        <v>1.647</v>
+        <v>2.125</v>
       </c>
       <c r="F65" t="n">
-        <v>2</v>
+        <v>2.042</v>
       </c>
       <c r="G65" t="n">
-        <v>0.353</v>
+        <v>-0.083</v>
       </c>
     </row>
     <row r="66">
@@ -12445,20 +12520,20 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>zh-Hant</t>
+          <t>zh-Hans</t>
         </is>
       </c>
       <c r="D66" t="n">
         <v>2</v>
       </c>
       <c r="E66" t="n">
-        <v>1.458</v>
+        <v>1.647</v>
       </c>
       <c r="F66" t="n">
         <v>2</v>
       </c>
       <c r="G66" t="n">
-        <v>0.542</v>
+        <v>0.353</v>
       </c>
     </row>
     <row r="67">
@@ -12469,25 +12544,25 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>T9</t>
+          <t>T6flip</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>zh-Hant</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E67" t="n">
-        <v>1.125</v>
+        <v>1.458</v>
       </c>
       <c r="F67" t="n">
-        <v>0.125</v>
+        <v>2</v>
       </c>
       <c r="G67" t="n">
-        <v>-1</v>
+        <v>0.542</v>
       </c>
     </row>
     <row r="68">
@@ -12503,20 +12578,20 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>zh-Hans</t>
+          <t>en</t>
         </is>
       </c>
       <c r="D68" t="n">
         <v>0</v>
       </c>
       <c r="E68" t="n">
-        <v>1.286</v>
+        <v>1.125</v>
       </c>
       <c r="F68" t="n">
-        <v>0.231</v>
+        <v>0.125</v>
       </c>
       <c r="G68" t="n">
-        <v>-1.055</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="69">
@@ -12532,19 +12607,48 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
+          <t>zh-Hans</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" t="n">
+        <v>1.286</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0.231</v>
+      </c>
+      <c r="G69" t="n">
+        <v>-1.055</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>gpt-5.5</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>T9</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
           <t>zh-Hant</t>
         </is>
       </c>
-      <c r="D69" t="n">
+      <c r="D70" t="n">
         <v>0.5</v>
       </c>
-      <c r="E69" t="n">
+      <c r="E70" t="n">
         <v>1.75</v>
       </c>
-      <c r="F69" t="n">
+      <c r="F70" t="n">
         <v>0.5</v>
       </c>
-      <c r="G69" t="n">
+      <c r="G70" t="n">
         <v>-1.25</v>
       </c>
     </row>

</xml_diff>